<commit_message>
feat: new horario export
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/templates/plantilla-horario.xlsx
+++ b/backend/src/main/resources/templates/plantilla-horario.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,27 +26,50 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00888888"/>
-      <sz val="8"/>
+      <color rgb="00999999"/>
+      <sz val="9"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00000000"/>
       <sz val="13"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
+      <color rgb="00000000"/>
       <sz val="9"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00000000"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -59,7 +82,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00B9BFC7"/>
       </patternFill>
     </fill>
     <fill>
@@ -104,37 +127,38 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -210,41 +234,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>prompt-export-horario</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Ancla para insertar el logo institucional (PNG) via POI ClientAnchor. Ocupa aprox. filas 1-4, columnas A-B. Reemplazar esta celda de placeholder por la imagen real.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>Ancla para insertar el logo de la especialidad (PNG, según CursoBase.especialidad) via POI ClientAnchor. Ocupa aprox. filas 1-4, columnas E-F.</t>
-      </text>
-    </comment>
-    <comment ref="A11" authorId="0" shapeId="0">
-      <text>
-        <t>Fila 'Salas': se agrega al final de cada bloque continuo de horas (sin receso en medio). Si la sala cambia entre horas del mismo bloque para el mismo día, concatenar valores con '/'.</t>
-      </text>
-    </comment>
-    <comment ref="A12" authorId="0" shapeId="0">
-      <text>
-        <t>Color de fondo PLACEHOLDER. En tiempo de generación, reemplazar el fgColor de este fill por el color HEX de la especialidad (extraído de frontend/src/index.css, :root[data-specialty="..."] { --accent: ... }).</t>
-      </text>
-    </comment>
-    <comment ref="A17" authorId="0" shapeId="0">
-      <text>
-        <t>Fila 'Salas': se agrega al final de cada bloque continuo de horas (sin receso en medio). Si la sala cambia entre horas del mismo bloque para el mismo día, concatenar valores con '/'.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -536,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -553,10 +542,10 @@
           <t>[LOGO INSTITUCIONAL]</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>HORARIO DE CLASES {{ANIO}}</t>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Ministerio de Educación y Ciencias
+Colegio Técnico Nacional</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -564,402 +553,416 @@
           <t>[LOGO ESPECIALIDAD]</t>
         </is>
       </c>
-      <c r="F1" s="2" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="4" t="inlineStr">
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Carga Horaria: 35 minutos</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Especialidad: {{ESPECIALIDAD}}</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Turno: {{TURNO}}</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="4" t="inlineStr">
+    </row>
+    <row r="5">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Sección: {{SECCION}}</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-    </row>
-    <row r="5" ht="6" customHeight="1"/>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Año: {{ANIO}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>{{NIVEL_LABEL}}</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Hora</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Martes</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Jueves</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Viernes</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>1°
 07:00 - 07:35</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="n"/>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>2°
 07:35 - 08:10</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="n"/>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="5" t="n"/>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Salas</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>{{SALA}}</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>{{SALA}}</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>{{SALA}}</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>{{SALA}}</t>
         </is>
       </c>
-      <c r="F11" s="11" t="inlineStr">
+      <c r="F12" s="10" t="inlineStr">
         <is>
           <t>{{SALA}}</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>RECESO</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>3°
 09:40 - 10:15</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="n"/>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="5" t="n"/>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>4°
 10:15 - 10:50</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>{{MATERIA}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="n"/>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>{{PROFESOR}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>{{MATERIA}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="5" t="n"/>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>{{PROFESOR}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Salas</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>{{SALA}}</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>{{SALA}}</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>{{SALA}}</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>{{SALA}}</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr">
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>{{SALA}}</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A12:F12"/>
+  <mergeCells count="10">
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="A1:B4"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="E1:F4"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A10:A11"/>
     <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="A14:A15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>